<commit_message>
initial action to transform json
</commit_message>
<xml_diff>
--- a/project/excel/include_schema.xlsx
+++ b/project/excel/include_schema.xlsx
@@ -1,30 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="17" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aliquot" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assay" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Biospecimen" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Condition" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DataFile" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FamilyGroup" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Participant" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Study" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thing" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Aliquot1" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assay1" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Biospecimen1" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Condition1" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DataFile1" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FamilyGroup1" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Participant1" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Study1" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thing1" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Aliquot" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Assay" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Biospecimen" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Condition" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="DataFile" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="FamilyGroup" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Participant" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Study" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Thing" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Aliquot1" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Assay1" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Biospecimen1" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Condition1" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="DataFile1" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="FamilyGroup1" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Participant1" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Study1" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Thing1" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -583,7 +583,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -645,6 +645,11 @@
       <c r="L1" t="inlineStr">
         <is>
           <t>other_code</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>neuron_type</t>
         </is>
       </c>
     </row>
@@ -1046,7 +1051,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:M1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1110,20 +1115,31 @@
           <t>other_code</t>
         </is>
       </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>neuron_type</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <dataValidations count="4">
+  <dataValidations count="6">
     <dataValidation sqref="E2:E1048576" showErrorMessage="1" showInputMessage="1" allowBlank="1" type="list">
       <formula1>"observed,not_observed"</formula1>
     </dataValidation>
     <dataValidation sqref="F2:F1048576" showErrorMessage="1" showInputMessage="1" allowBlank="1" type="list">
       <formula1>"clinical,self_reported"</formula1>
     </dataValidation>
+    <dataValidation sqref="M2:M1048576" showErrorMessage="1" showInputMessage="1" allowBlank="1" type="list">
+      <formula1>""</formula1>
+    </dataValidation>
     <dataValidation sqref="E2:E1048576" showErrorMessage="1" showInputMessage="1" allowBlank="1" type="list">
       <formula1>"observed,not_observed"</formula1>
     </dataValidation>
     <dataValidation sqref="F2:F1048576" showErrorMessage="1" showInputMessage="1" allowBlank="1" type="list">
       <formula1>"clinical,self_reported"</formula1>
+    </dataValidation>
+    <dataValidation sqref="M2:M1048576" showErrorMessage="1" showInputMessage="1" allowBlank="1" type="list">
+      <formula1>""</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>